<commit_message>
Release v1.1.0: cleaned PSTE code verified against the code used in the revised manuscript (restore planning reserve margin, align solver settings and cost terms), correct README, add configs, licence and provenance
</commit_message>
<xml_diff>
--- a/data/energy_story_2020.xlsx
+++ b/data/energy_story_2020.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\paper2\data\Power_generate\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{618EDB01-05E8-4195-8C8F-061CB964E88B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>